<commit_message>
Feat: Creacion de pedidos, Creacion de configuraciones
</commit_message>
<xml_diff>
--- a/app/features/process_shipment/filleo/templates/formato-envio.xlsx
+++ b/app/features/process_shipment/filleo/templates/formato-envio.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" state="veryHidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="999999" calcMode="auto" fullCalcOnLoad="1" calcCompleted="0"/>
 </workbook>
 </file>
 
@@ -20,13 +20,15 @@
   <fonts count="2">
     <font>
       <name val="Calibri"/>
+      <strike val="0"/>
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
+      <strike val="0"/>
+      <color rgb="FFffffff"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -35,48 +37,49 @@
       <patternFill/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0076FA"/>
+        <fgColor rgb="FF0076fa"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -439,17 +442,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N500"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:N501"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="5" min="1" max="1"/>
     <col width="25" customWidth="1" style="5" min="2" max="2"/>
     <col width="20" customWidth="1" style="5" min="3" max="3"/>
     <col width="25" customWidth="1" style="5" min="4" max="4"/>
     <col width="20" customWidth="1" style="5" min="5" max="5"/>
-    <col width="30" customWidth="1" style="5" min="6" max="7"/>
+    <col width="30" customWidth="1" style="5" min="6" max="6"/>
+    <col width="30" customWidth="1" style="5" min="7" max="7"/>
     <col width="15" customWidth="1" style="5" min="8" max="8"/>
-    <col width="10" customWidth="1" style="5" min="9" max="12"/>
+    <col width="10" customWidth="1" style="5" min="9" max="9"/>
+    <col width="10" customWidth="1" style="5" min="10" max="10"/>
+    <col width="10" customWidth="1" style="5" min="11" max="11"/>
+    <col width="10" customWidth="1" style="5" min="12" max="12"/>
     <col width="11" customWidth="1" style="5" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -526,7 +533,7 @@
         <v>70951063</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>123456789</v>
+        <v>921584492</v>
       </c>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
@@ -538,7 +545,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>QUILLABAMBA</t>
+          <t>AV  JOSE GALVEZ</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -8032,13 +8039,4525 @@
       <c r="L500" s="2" t="n"/>
       <c r="M500" s="2" t="n"/>
     </row>
+    <row r="501">
+      <c r="F501" s="0" t="n"/>
+      <c r="G501" s="0" t="n"/>
+      <c r="H501" s="0" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+  <dataValidations count="1500">
+    <dataValidation sqref="F2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F93" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G93" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H93" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F95" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G95" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H95" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F111" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G111" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H111" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F116" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G116" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H116" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F123" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G123" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H123" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F128" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G128" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H128" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F132" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G132" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H132" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F133" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G133" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H133" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F136" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G136" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H136" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F144" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G144" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H144" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F145" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G145" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H145" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F149" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G149" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H149" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F150" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G150" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H150" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F152" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G152" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H152" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F153" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G153" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H153" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F154" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G154" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H154" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F155" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G155" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H155" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F157" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G157" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H157" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F159" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G159" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H159" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F160" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G160" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H160" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F162" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G162" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H162" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F164" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G164" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H164" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F165" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G165" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H165" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F166" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G166" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H166" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F168" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G168" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H168" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F169" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G169" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H169" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F170" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G170" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H170" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F172" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G172" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H172" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F173" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G173" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H173" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F174" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G174" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H174" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F176" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G176" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H176" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F177" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G177" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H177" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F178" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G178" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H178" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F179" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G179" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H179" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F180" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G180" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H180" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F184" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G184" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H184" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F185" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G185" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H185" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F187" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G187" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H187" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F188" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G188" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H188" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F189" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G189" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H189" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F190" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G190" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H190" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F191" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G191" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H191" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F192" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G192" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H192" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F193" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G193" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H193" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F194" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G194" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H194" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F195" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G195" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H195" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F196" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G196" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H196" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F197" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G197" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H197" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F198" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G198" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H198" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F199" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G199" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H199" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F202" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G202" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H202" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F205" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G205" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H205" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F206" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G206" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H206" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F207" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G207" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H207" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F208" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G208" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H208" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F209" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G209" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H209" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F211" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G211" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H211" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F213" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G213" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H213" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F214" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G214" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H214" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F215" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G215" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H215" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F216" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G216" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H216" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F217" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G217" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H217" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F218" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G218" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H218" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F219" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G219" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H219" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F220" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G220" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H220" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F221" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G221" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H221" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F222" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G222" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H222" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F223" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G223" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H223" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F224" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G224" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H224" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F226" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G226" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H226" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F227" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G227" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H227" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F228" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G228" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H228" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F229" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G229" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H229" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F230" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G230" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H230" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F231" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G231" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H231" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F232" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G232" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H232" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F233" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G233" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H233" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F234" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G234" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H234" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F235" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G235" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H235" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F236" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G236" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H236" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F237" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G237" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H237" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F238" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G238" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H238" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F239" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G239" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H239" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F240" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G240" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H240" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F241" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G241" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H241" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F242" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G242" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H242" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F243" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G243" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H243" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F244" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G244" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H244" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F245" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G245" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H245" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F246" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G246" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H246" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F247" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G247" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H247" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F248" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G248" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H248" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F249" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G249" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H249" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F250" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G250" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H250" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F251" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G251" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H251" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F252" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G252" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H252" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F253" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G253" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H253" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F254" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G254" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H254" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F255" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G255" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H255" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F256" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G256" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H256" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H257" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H258" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F259" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G259" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H259" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F260" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G260" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H260" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F261" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G261" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H261" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F262" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G262" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H262" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F263" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G263" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H263" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F264" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G264" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H264" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F265" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G265" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H265" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F266" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G266" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H266" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F267" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G267" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H267" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F268" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G268" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H268" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F269" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G269" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H269" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F270" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G270" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H270" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F271" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G271" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H271" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F272" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G272" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H272" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F273" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G273" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H273" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F274" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G274" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H274" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F275" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G275" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H275" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F276" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G276" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H276" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F277" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G277" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H277" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F278" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G278" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H278" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F279" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G279" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H279" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F280" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G280" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H280" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F281" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G281" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H281" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F282" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G282" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H282" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F283" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G283" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H283" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F284" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G284" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H284" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F285" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G285" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H285" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F286" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G286" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H286" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F287" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G287" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H287" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F288" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G288" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H288" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F289" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G289" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H289" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F290" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G290" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H290" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F291" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G291" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H291" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F292" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G292" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H292" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F293" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G293" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H293" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F294" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G294" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H294" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F295" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G295" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H295" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F296" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G296" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H296" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F297" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G297" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H297" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F298" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G298" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H298" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F299" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G299" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H299" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F302" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G302" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H302" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F303" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G303" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H303" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F305" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G305" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H305" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F306" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G306" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H306" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F307" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G307" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H307" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F308" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G308" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H308" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F309" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G309" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H309" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F310" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G310" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H310" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F311" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G311" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H311" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F312" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G312" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H312" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F313" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G313" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H313" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F314" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G314" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H314" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F315" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G315" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H315" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F316" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G316" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H316" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F317" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G317" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H317" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F318" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G318" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H318" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F319" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G319" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H319" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F320" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G320" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H320" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F321" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G321" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H321" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F322" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G322" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H322" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F323" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G323" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H323" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F324" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G324" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H324" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F325" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G325" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H325" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F326" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G326" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H326" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F327" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G327" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H327" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F328" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G328" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H328" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F329" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G329" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H329" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F330" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G330" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H330" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F331" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G331" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H331" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F332" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G332" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H332" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F333" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G333" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H333" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F334" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G334" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H334" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F335" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G335" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H335" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F336" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G336" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H336" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F337" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G337" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H337" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F338" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G338" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H338" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F339" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G339" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H339" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F340" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G340" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H340" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F342" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G342" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H342" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F343" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G343" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H343" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F344" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G344" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H344" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F345" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G345" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H345" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F346" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G346" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H346" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F347" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G347" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H347" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F348" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G348" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H348" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F349" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G349" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H349" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F350" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G350" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H350" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F351" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G351" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H351" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F352" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G352" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H352" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F353" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G353" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H353" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F354" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G354" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H354" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F355" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G355" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H355" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F356" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G356" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H356" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F357" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G357" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H357" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F358" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G358" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H358" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F359" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G359" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H359" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F360" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G360" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H360" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F361" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G361" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H361" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F362" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G362" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H362" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F363" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G363" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H363" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F364" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G364" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H364" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F365" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G365" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H365" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F366" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G366" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H366" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F367" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G367" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H367" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F368" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G368" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H368" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F369" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G369" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H369" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F370" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G370" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H370" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F371" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G371" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H371" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F372" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G372" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H372" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F373" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G373" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H373" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F374" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G374" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H374" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F375" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G375" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H375" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F376" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G376" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H376" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F377" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G377" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H377" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F378" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G378" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H378" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F379" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G379" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H379" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F380" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G380" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H380" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F381" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G381" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H381" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F382" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G382" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H382" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F383" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G383" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H383" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F384" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G384" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H384" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F385" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G385" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H385" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F386" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G386" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H386" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F387" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G387" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H387" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F388" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G388" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H388" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F389" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G389" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H389" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F390" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G390" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H390" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F391" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G391" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H391" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F392" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G392" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H392" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F393" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G393" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H393" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F394" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G394" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H394" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F395" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G395" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H395" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F396" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G396" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H396" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F397" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G397" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H397" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F398" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G398" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H398" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F399" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G399" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H399" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F401" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G401" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H401" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F402" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G402" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H402" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F403" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G403" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H403" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F404" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G404" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H404" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F405" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G405" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H405" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F406" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G406" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H406" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F407" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G407" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H407" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F408" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G408" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H408" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F409" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G409" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H409" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F410" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G410" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H410" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F411" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G411" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H411" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F412" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G412" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H412" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F413" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G413" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H413" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F414" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G414" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H414" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F415" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G415" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H415" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F416" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G416" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H416" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F417" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G417" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H417" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F418" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G418" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H418" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F419" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G419" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H419" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F420" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G420" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H420" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F421" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G421" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H421" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F422" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G422" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H422" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F423" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G423" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H423" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F424" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G424" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H424" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F425" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G425" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H425" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F426" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G426" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H426" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F427" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G427" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H427" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F428" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G428" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H428" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F429" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G429" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H429" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F430" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G430" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H430" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F431" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G431" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H431" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F432" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G432" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H432" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F433" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G433" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H433" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F434" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G434" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H434" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F435" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G435" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H435" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F436" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G436" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H436" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F437" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G437" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H437" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F438" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G438" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H438" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F439" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G439" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H439" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F440" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G440" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H440" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F441" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G441" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H441" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F442" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G442" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H442" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F443" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G443" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H443" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F444" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G444" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H444" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F445" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G445" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H445" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F446" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G446" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H446" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F447" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G447" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H447" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F448" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G448" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H448" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F449" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G449" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H449" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F450" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G450" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H450" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F451" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G451" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H451" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F452" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G452" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H452" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F453" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G453" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H453" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F454" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G454" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H454" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F455" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G455" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H455" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F456" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G456" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H456" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F457" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G457" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H457" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F458" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G458" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H458" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F459" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G459" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H459" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F460" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G460" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H460" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F461" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G461" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H461" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F462" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G462" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H462" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F463" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G463" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H463" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F464" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G464" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H464" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F465" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G465" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H465" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F466" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G466" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H466" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F467" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G467" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H467" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F468" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G468" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H468" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F469" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G469" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H469" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F470" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G470" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H470" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F471" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G471" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H471" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F472" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G472" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H472" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F473" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G473" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H473" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F474" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G474" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H474" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F475" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G475" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H475" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F476" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G476" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H476" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F477" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G477" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H477" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F478" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G478" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H478" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F479" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G479" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H479" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F480" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G480" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H480" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F481" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G481" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H481" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F482" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G482" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H482" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F483" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G483" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H483" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F484" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G484" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H484" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F485" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G485" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H485" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F486" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G486" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H486" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F487" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G487" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H487" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F488" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G488" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H488" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F489" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G489" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H489" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F490" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G490" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H490" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F491" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G491" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H491" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F492" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G492" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H492" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F493" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G493" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H493" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F494" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G494" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H494" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F495" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G495" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H495" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F496" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G496" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H496" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F497" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G497" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H497" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F498" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G498" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H498" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F499" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G499" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H499" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$B$2:$B$482</formula1>
+    </dataValidation>
+    <dataValidation sqref="G501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
+      <formula1>'Hoja2'!$C$2:$C$468</formula1>
+    </dataValidation>
+    <dataValidation sqref="H501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Error de escritura" error="Valor fuera de lista" type="list" errorStyle="information">
       <formula1>"SOBRE,PAQUETE XXS,PAQUETE XS,PAQUETE S,PAQUETE M,PAQUETE L,CAJA,BULTO"</formula1>
     </dataValidation>
   </dataValidations>
+  <printOptions gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="default" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="1" alignWithMargins="1">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -8049,10 +12568,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G1685"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <cols>
-    <col width="40" customWidth="1" style="5" min="2" max="3"/>
-    <col width="25" customWidth="1" style="5" min="4" max="9"/>
+    <col width="40" customWidth="1" style="5" min="2" max="2"/>
+    <col width="40" customWidth="1" style="5" min="3" max="3"/>
+    <col width="25" customWidth="1" style="5" min="4" max="4"/>
+    <col width="25" customWidth="1" style="5" min="5" max="5"/>
+    <col width="25" customWidth="1" style="5" min="6" max="6"/>
+    <col width="25" customWidth="1" style="5" min="7" max="7"/>
+    <col width="25" customWidth="1" style="5" min="8" max="8"/>
+    <col width="25" customWidth="1" style="5" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -27139,6 +31664,16 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="default" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="1" alignWithMargins="1">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Feat: Envio de codigo ahora es por pedido
</commit_message>
<xml_diff>
--- a/app/features/process_shipment/filleo/templates/formato-envio.xlsx
+++ b/app/features/process_shipment/filleo/templates/formato-envio.xlsx
@@ -533,7 +533,7 @@
         <v>70951063</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>921584492</v>
+        <v>987654321</v>
       </c>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
@@ -545,7 +545,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>AV  JOSE GALVEZ</t>
+          <t>AV  J GALVEZ</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">

</xml_diff>